<commit_message>
Publish PR preview pr-51
</commit_message>
<xml_diff>
--- a/pr-preview/pr-51/obyvak-skladba-materialu.xlsx
+++ b/pr-preview/pr-51/obyvak-skladba-materialu.xlsx
@@ -793,56 +793,60 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="52" customHeight="1">
-      <c r="A6" s="4" t="n">
+    <row r="6" ht="44" customHeight="1">
+      <c r="A6" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Parozábrana</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Parotěsná fólie</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Výrobek dosud nezvolen</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>≈ 1 mm (model)</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="n">
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Reflexní parozábrana Al</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Jutafol 145 Al (JUTA; retail N AL 170 Speciál 75 m²)</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Al reflex · Sd vysoké · role 1,5×50 m</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="n">
         <v>71</v>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="H6" s="9" t="inlineStr">
         <is>
           <t>10 %</t>
         </is>
       </c>
-      <c r="I6" s="6" t="n">
+      <c r="I6" s="9" t="n">
         <v>78.09999999999999</v>
       </c>
-      <c r="J6" s="6" t="n"/>
-      <c r="K6" s="6" t="n"/>
-      <c r="L6" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M6" s="4" t="inlineStr">
-        <is>
-          <t>Nedořešeno: typ / Sd / systém pásek.</t>
+      <c r="J6" s="10" t="n">
+        <v>35.73</v>
+      </c>
+      <c r="K6" s="11" t="n">
+        <v>2791</v>
+      </c>
+      <c r="L6" s="7" t="inlineStr">
+        <is>
+          <t>IZOMAT JUTAFOL N AL 170 Speciál · https://www.izomat.cz/parozabrana-juta-jutafol-n-al-170-special.html</t>
+        </is>
+      </c>
+      <c r="M6" s="7" t="inlineStr">
+        <is>
+          <t>Na attic straně CD, pod minerální vlnou (stejně jako zbytek domu — ne proměnlivá fólie). Plocha šikmin 71.00 m². S rezervou 10 % ≈ 78.1 m² ≈ 2× role 75 m². Přesahy: JUTAFOL SP AL / SP 1.</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1268,7 @@
       <c r="I15" s="15" t="n"/>
       <c r="J15" s="15" t="n"/>
       <c r="K15" s="16" t="n">
-        <v>58179</v>
+        <v>60970</v>
       </c>
       <c r="L15" s="15" t="n"/>
       <c r="M15" s="15" t="n"/>
@@ -1272,7 +1276,7 @@
     <row r="16" ht="36" customHeight="1">
       <c r="A16" s="17" t="inlineStr">
         <is>
-          <t>Neoceněno (chybí v součtu): Povrchová úprava; Podkladní nátěr; Parozábrana; Výplň dutiny / mezi krokvemi; Krov (nosná konstrukce)</t>
+          <t>Neoceněno (chybí v součtu): Povrchová úprava; Podkladní nátěr; Výplň dutiny / mezi krokvemi; Krov (nosná konstrukce)</t>
         </is>
       </c>
       <c r="B16" s="18" t="n"/>
@@ -1299,10 +1303,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1716,7 +1721,7 @@
         </is>
       </c>
       <c r="F8" s="9" t="n">
-        <v>5.76</v>
+        <v>5.78</v>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
@@ -1729,13 +1734,13 @@
         </is>
       </c>
       <c r="I8" s="9" t="n">
-        <v>6.46</v>
+        <v>6.47</v>
       </c>
       <c r="J8" s="10" t="n">
         <v>115.88</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>748</v>
+        <v>750</v>
       </c>
       <c r="L8" s="7" t="inlineStr">
         <is>
@@ -2178,7 +2183,7 @@
       <c r="I17" s="15" t="n"/>
       <c r="J17" s="15" t="n"/>
       <c r="K17" s="16" t="n">
-        <v>16625</v>
+        <v>16627</v>
       </c>
       <c r="L17" s="15" t="n"/>
       <c r="M17" s="15" t="n"/>
@@ -3071,56 +3076,60 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="52" customHeight="1">
-      <c r="A7" s="4" t="n">
+    <row r="7" ht="44" customHeight="1">
+      <c r="A7" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Parozábrana</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Fólie</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Výrobek dosud nezvolen</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="n">
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Jutafol 145 Al</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Jutafol 145 Al</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>role 75 m²</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="n">
         <v>71</v>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="H7" s="9" t="inlineStr">
         <is>
           <t>10 %</t>
         </is>
       </c>
-      <c r="I7" s="6" t="n">
+      <c r="I7" s="9" t="n">
         <v>78.09999999999999</v>
       </c>
-      <c r="J7" s="6" t="n"/>
-      <c r="K7" s="6" t="n"/>
-      <c r="L7" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M7" s="4" t="inlineStr">
-        <is>
-          <t>Nedořešeno.</t>
+      <c r="J7" s="10" t="n">
+        <v>35.73</v>
+      </c>
+      <c r="K7" s="11" t="n">
+        <v>2791</v>
+      </c>
+      <c r="L7" s="7" t="inlineStr">
+        <is>
+          <t>IZOMAT JUTAFOL N AL 170 Speciál · https://www.izomat.cz/parozabrana-juta-jutafol-n-al-170-special.html</t>
+        </is>
+      </c>
+      <c r="M7" s="7" t="inlineStr">
+        <is>
+          <t>Šikminy 71.00 m² (+10 % ≈ 78.1 m²). Nad CD, pod vlnou.</t>
         </is>
       </c>
     </row>
@@ -3149,7 +3158,7 @@
         </is>
       </c>
       <c r="F8" s="9" t="n">
-        <v>76.76000000000001</v>
+        <v>76.78</v>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
@@ -3162,13 +3171,13 @@
         </is>
       </c>
       <c r="I8" s="9" t="n">
-        <v>85.98</v>
+        <v>85.98999999999999</v>
       </c>
       <c r="J8" s="10" t="n">
         <v>115.88</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>9963</v>
+        <v>9965</v>
       </c>
       <c r="L8" s="7" t="inlineStr">
         <is>
@@ -3892,7 +3901,7 @@
       <c r="I22" s="15" t="n"/>
       <c r="J22" s="15" t="n"/>
       <c r="K22" s="16" t="n">
-        <v>102909</v>
+        <v>105702</v>
       </c>
       <c r="L22" s="15" t="n"/>
       <c r="M22" s="15" t="n"/>
@@ -3900,7 +3909,7 @@
     <row r="23" ht="36" customHeight="1">
       <c r="A23" s="17" t="inlineStr">
         <is>
-          <t>Neoceněno (chybí v součtu): StoSilent Top Finish; StoSilent Top Basic; Parozábrana; Minerální vlna (souhrn)</t>
+          <t>Neoceněno (chybí v součtu): StoSilent Top Finish; StoSilent Top Basic; Minerální vlna (souhrn)</t>
         </is>
       </c>
       <c r="B23" s="18" t="n"/>
@@ -3928,12 +3937,13 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>